<commit_message>
removing The 1 year in SOPs
</commit_message>
<xml_diff>
--- a/Matar Trainings.xlsx
+++ b/Matar Trainings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\l.karuru\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F4B6E8-5257-4DA6-B5C5-344DFDF46082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CD39485-1A96-4935-9C1E-FBE5787DA781}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{2ACD8935-9A55-49F4-8AD3-9F8021E2249D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2ACD8935-9A55-49F4-8AD3-9F8021E2249D}"/>
   </bookViews>
   <sheets>
     <sheet name="Meta Data" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1658" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1665" uniqueCount="513">
   <si>
     <t>Emp. No.</t>
   </si>
@@ -1240,331 +1240,334 @@
     <t>Mark Merill Jovenes Tirol</t>
   </si>
   <si>
+    <t>Francis Agbor Eyong Atem</t>
+  </si>
+  <si>
+    <t>Siraj Moolakkappil</t>
+  </si>
+  <si>
+    <t>Mohamed Bilal Muneer Basha</t>
+  </si>
+  <si>
+    <t>Alen Cherippanat Babu</t>
+  </si>
+  <si>
+    <t>Mohamed Shafras Jawlangull</t>
+  </si>
+  <si>
+    <t>Renson Gicheha Gicheru</t>
+  </si>
+  <si>
+    <t>Mohamed Faris Mohamed Naleem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shihabdeen Seeni Mohamed </t>
+  </si>
+  <si>
+    <t>Prakyath Prabhakar Amin</t>
+  </si>
+  <si>
+    <t>Julius Kateregga</t>
+  </si>
+  <si>
+    <t>Kishanraj Pulenthiran</t>
+  </si>
+  <si>
+    <t>James Kariungi Muthee</t>
+  </si>
+  <si>
+    <t>Kasansula Francis Kiwanuka</t>
+  </si>
+  <si>
+    <t>Arnel Neri Montemayor</t>
+  </si>
+  <si>
+    <t>Erick Omondi Okoyo</t>
+  </si>
+  <si>
+    <t>Trevin Christopher Neydorf</t>
+  </si>
+  <si>
+    <t>Mohamed Mufaris Mohamed Jameel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jasim Kinarullaparambath Kunhabdulla </t>
+  </si>
+  <si>
+    <t>Naser Qasim Mohammad Alhaj Ahmed</t>
+  </si>
+  <si>
+    <t>Jeffrey Sayson Bagatua</t>
+  </si>
+  <si>
+    <t>Wali Mohammed Sabry</t>
+  </si>
+  <si>
+    <t>Rommel Tamayo Eleosida</t>
+  </si>
+  <si>
+    <t>Errolnil Purificacion Atienza</t>
+  </si>
+  <si>
+    <t>Hernan John Baguion Murcillos</t>
+  </si>
+  <si>
+    <t>Ivan Raphael Macatangay Del Mundo</t>
+  </si>
+  <si>
+    <t>Jerico Tallorin Atienzo</t>
+  </si>
+  <si>
+    <t>Alvin Tumboc Cuevas</t>
+  </si>
+  <si>
+    <t>James Andrew Aquino Rodillo</t>
+  </si>
+  <si>
+    <t>Alvin Cataquiz Austria</t>
+  </si>
+  <si>
+    <t>Jayson Ruz Oligan</t>
+  </si>
+  <si>
+    <t>John Michael Angelo Mesina Clemen</t>
+  </si>
+  <si>
+    <t>Lemuel Carcellar Macatangay</t>
+  </si>
+  <si>
+    <t>Nikko Villanueva Cruz</t>
+  </si>
+  <si>
+    <t>Justin Paolo Macatangay Ilao</t>
+  </si>
+  <si>
+    <t>Jake Alinabon Salibay</t>
+  </si>
+  <si>
+    <t>Marlon Yuson Pamplona</t>
+  </si>
+  <si>
+    <t>Joe Vergil Jr Calanza Dormitorio</t>
+  </si>
+  <si>
+    <t>Bonifacio Arano Bayer</t>
+  </si>
+  <si>
+    <t>Sumedha Pradeep Dissanayaka</t>
+  </si>
+  <si>
+    <t>Yuvashanth Somasuntharam kukasuthan</t>
+  </si>
+  <si>
+    <t>Jonel Catibog Katigbak</t>
+  </si>
+  <si>
+    <t>Catalino Mendoza Rojas</t>
+  </si>
+  <si>
+    <t>Murshidul Haq Patteri Thazhe Kuni</t>
+  </si>
+  <si>
+    <t>Nisham Kizhakke Valappil</t>
+  </si>
+  <si>
+    <t>Pasidu Pamodaya Rathnayake Rathnayake Mudiyanselage</t>
+  </si>
+  <si>
+    <t>Chalana Ishan Dishanayake Dishanayake Pathiranage</t>
+  </si>
+  <si>
+    <t>Mohamed Ahthir Abdul Majeed</t>
+  </si>
+  <si>
+    <t>Niroshan Abesingha Abesingha Karunarathna Mudalige</t>
+  </si>
+  <si>
+    <t>Sathis Gunawardhana Dikella Kandha Yakdhehirallage</t>
+  </si>
+  <si>
+    <t>Tharaka Thanujaya Dissanayaka Dissanayaka Mudiyanselage</t>
+  </si>
+  <si>
+    <t>Nishan Ekanayake Ekanayake Mudiyanselage</t>
+  </si>
+  <si>
+    <t>Jacky Chan Nava Gastardo</t>
+  </si>
+  <si>
+    <t>Mohammed Fahim Mohammed Laffir</t>
+  </si>
+  <si>
+    <t>Sameera Lakmal Rupasinghe Arachchige</t>
+  </si>
+  <si>
+    <t>Dushan Priyankara Herath Herath Mudiyanselage</t>
+  </si>
+  <si>
+    <t>Pathmapriyan Muruguppilla</t>
+  </si>
+  <si>
+    <t>Roshan Chaminda Udawaththa Udawaththa Kankanamge</t>
+  </si>
+  <si>
+    <t>Kusal Sharmila Hewa Kokawalage</t>
+  </si>
+  <si>
+    <t>Mohomed Minnas Mohomed Ramees</t>
+  </si>
+  <si>
+    <t>Mabin Pauly</t>
+  </si>
+  <si>
+    <t>Jahsim Saycon Apila</t>
+  </si>
+  <si>
+    <t>Shern Sebastian Sebastian Simon</t>
+  </si>
+  <si>
+    <t>Wai Hin Phyo</t>
+  </si>
+  <si>
+    <t>Hicham Charkaoui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mohamed Shaheer Mohamed Laffir </t>
+  </si>
+  <si>
+    <t>Antony Kamau Kageche</t>
+  </si>
+  <si>
+    <t>Abdulrashid Byarugaba </t>
+  </si>
+  <si>
+    <t>Justine Tiangson Clave</t>
+  </si>
+  <si>
+    <t>Harikaran Seenithamby</t>
+  </si>
+  <si>
+    <t>Wycliffe Mushori</t>
+  </si>
+  <si>
+    <t>Peter Nganga Kamau</t>
+  </si>
+  <si>
+    <t>Sumesh Soman</t>
+  </si>
+  <si>
+    <t>Muhammed Ashiq Mohamed Mumtaz</t>
+  </si>
+  <si>
+    <t>Arvin Clyde D.Crisme</t>
+  </si>
+  <si>
+    <t>Gary John Packer</t>
+  </si>
+  <si>
+    <t>Ifras Mohammed</t>
+  </si>
+  <si>
+    <t>Alby Manchandiyil Antony</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ifran Ansari </t>
+  </si>
+  <si>
+    <t>Piratheepan Thiyagarasa</t>
+  </si>
+  <si>
+    <t>Moustafa Hassan Ibrahim Elsayyad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harsha Shetty </t>
+  </si>
+  <si>
+    <t>Kevin Carl Enriquez Serrano</t>
+  </si>
+  <si>
+    <t>Romie Ross Tamayo Eleosida</t>
+  </si>
+  <si>
+    <t>Quennan Carandang Cuesta</t>
+  </si>
+  <si>
+    <t>Lester John Fuentes Monter</t>
+  </si>
+  <si>
+    <t>Neil Jhon Sabile Ramos</t>
+  </si>
+  <si>
+    <t>Kim Harvey Cuevas Ayag</t>
+  </si>
+  <si>
+    <t>Nelson Jr Ybut Sancho</t>
+  </si>
+  <si>
+    <t>Rolly Miano Valdez</t>
+  </si>
+  <si>
+    <t>Daniel Bacolcol Orquiza</t>
+  </si>
+  <si>
+    <t>Roby Chua Malinao</t>
+  </si>
+  <si>
+    <t>Lorence Cardenas Cabales</t>
+  </si>
+  <si>
+    <t>Emmanuel Richard Marasigan Velasco</t>
+  </si>
+  <si>
+    <t>Michael Jorge Toscano Masaoy</t>
+  </si>
+  <si>
+    <t>Jeffrey De Vera Cabico</t>
+  </si>
+  <si>
+    <t>Joe Peter Angustia Pimentel</t>
+  </si>
+  <si>
+    <t>Mark Roentgen Macatangay Delen</t>
+  </si>
+  <si>
+    <t>Arjay Imperial Gabarda</t>
+  </si>
+  <si>
+    <t>Noey Francisco Canonizado</t>
+  </si>
+  <si>
+    <t>Omar Zaki Saad Abdel Nabi</t>
+  </si>
+  <si>
+    <t>Abdul Rehman Mohammed Abdul Mohammed</t>
+  </si>
+  <si>
+    <t>Christian Merck Morada Martija</t>
+  </si>
+  <si>
+    <t>Imesha Rashmi Mudannayaka Mudannayakage</t>
+  </si>
+  <si>
+    <t>Sajith Dulanjana Kumara Rathnayaka Mudiyanselage</t>
+  </si>
+  <si>
+    <t>Thisura Kaumal Wijesinghe</t>
+  </si>
+  <si>
+    <t>Shanel Rukshan Perera Kurana Patabendige</t>
+  </si>
+  <si>
+    <t>Abeykoon Mudiyanselage Sasitha Dinushka Abeykoon</t>
+  </si>
+  <si>
+    <t>Jerusha Anns Philip</t>
+  </si>
+  <si>
     <t>Kennedy Gichuhi Ngaruiya</t>
   </si>
   <si>
-    <t>Francis Agbor Eyong Atem</t>
-  </si>
-  <si>
-    <t>Siraj Moolakkappil</t>
-  </si>
-  <si>
-    <t>Mohamed Bilal Muneer Basha</t>
-  </si>
-  <si>
-    <t>Alen Cherippanat Babu</t>
-  </si>
-  <si>
-    <t>Mohamed Shafras Jawlangull</t>
-  </si>
-  <si>
-    <t>Renson Gicheha Gicheru</t>
-  </si>
-  <si>
-    <t>Mohamed Faris Mohamed Naleem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shihabdeen Seeni Mohamed </t>
-  </si>
-  <si>
-    <t>Prakyath Prabhakar Amin</t>
-  </si>
-  <si>
-    <t>Julius Kateregga</t>
-  </si>
-  <si>
-    <t>Kishanraj Pulenthiran</t>
-  </si>
-  <si>
-    <t>James Kariungi Muthee</t>
-  </si>
-  <si>
-    <t>Kasansula Francis Kiwanuka</t>
-  </si>
-  <si>
-    <t>Arnel Neri Montemayor</t>
-  </si>
-  <si>
-    <t>Erick Omondi Okoyo</t>
-  </si>
-  <si>
-    <t>Trevin Christopher Neydorf</t>
-  </si>
-  <si>
-    <t>Mohamed Mufaris Mohamed Jameel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jasim Kinarullaparambath Kunhabdulla </t>
-  </si>
-  <si>
-    <t>Naser Qasim Mohammad Alhaj Ahmed</t>
-  </si>
-  <si>
-    <t>Jeffrey Sayson Bagatua</t>
-  </si>
-  <si>
-    <t>Wali Mohammed Sabry</t>
-  </si>
-  <si>
-    <t>Rommel Tamayo Eleosida</t>
-  </si>
-  <si>
-    <t>Errolnil Purificacion Atienza</t>
-  </si>
-  <si>
-    <t>Hernan John Baguion Murcillos</t>
-  </si>
-  <si>
-    <t>Ivan Raphael Macatangay Del Mundo</t>
-  </si>
-  <si>
-    <t>Jerico Tallorin Atienzo</t>
-  </si>
-  <si>
-    <t>Alvin Tumboc Cuevas</t>
-  </si>
-  <si>
-    <t>James Andrew Aquino Rodillo</t>
-  </si>
-  <si>
-    <t>Alvin Cataquiz Austria</t>
-  </si>
-  <si>
-    <t>Jayson Ruz Oligan</t>
-  </si>
-  <si>
-    <t>John Michael Angelo Mesina Clemen</t>
-  </si>
-  <si>
-    <t>Lemuel Carcellar Macatangay</t>
-  </si>
-  <si>
-    <t>Nikko Villanueva Cruz</t>
-  </si>
-  <si>
-    <t>Justin Paolo Macatangay Ilao</t>
-  </si>
-  <si>
-    <t>Jake Alinabon Salibay</t>
-  </si>
-  <si>
-    <t>Marlon Yuson Pamplona</t>
-  </si>
-  <si>
-    <t>Joe Vergil Jr Calanza Dormitorio</t>
-  </si>
-  <si>
-    <t>Bonifacio Arano Bayer</t>
-  </si>
-  <si>
-    <t>Sumedha Pradeep Dissanayaka</t>
-  </si>
-  <si>
-    <t>Yuvashanth Somasuntharam kukasuthan</t>
-  </si>
-  <si>
-    <t>Jonel Catibog Katigbak</t>
-  </si>
-  <si>
-    <t>Catalino Mendoza Rojas</t>
-  </si>
-  <si>
-    <t>Murshidul Haq Patteri Thazhe Kuni</t>
-  </si>
-  <si>
-    <t>Nisham Kizhakke Valappil</t>
-  </si>
-  <si>
-    <t>Pasidu Pamodaya Rathnayake Rathnayake Mudiyanselage</t>
-  </si>
-  <si>
-    <t>Chalana Ishan Dishanayake Dishanayake Pathiranage</t>
-  </si>
-  <si>
-    <t>Mohamed Ahthir Abdul Majeed</t>
-  </si>
-  <si>
-    <t>Niroshan Abesingha Abesingha Karunarathna Mudalige</t>
-  </si>
-  <si>
-    <t>Sathis Gunawardhana Dikella Kandha Yakdhehirallage</t>
-  </si>
-  <si>
-    <t>Tharaka Thanujaya Dissanayaka Dissanayaka Mudiyanselage</t>
-  </si>
-  <si>
-    <t>Nishan Ekanayake Ekanayake Mudiyanselage</t>
-  </si>
-  <si>
-    <t>Jacky Chan Nava Gastardo</t>
-  </si>
-  <si>
-    <t>Mohammed Fahim Mohammed Laffir</t>
-  </si>
-  <si>
-    <t>Sameera Lakmal Rupasinghe Arachchige</t>
-  </si>
-  <si>
-    <t>Dushan Priyankara Herath Herath Mudiyanselage</t>
-  </si>
-  <si>
-    <t>Pathmapriyan Muruguppilla</t>
-  </si>
-  <si>
-    <t>Roshan Chaminda Udawaththa Udawaththa Kankanamge</t>
-  </si>
-  <si>
-    <t>Kusal Sharmila Hewa Kokawalage</t>
-  </si>
-  <si>
-    <t>Mohomed Minnas Mohomed Ramees</t>
-  </si>
-  <si>
-    <t>Mabin Pauly</t>
-  </si>
-  <si>
-    <t>Jahsim Saycon Apila</t>
-  </si>
-  <si>
-    <t>Shern Sebastian Sebastian Simon</t>
-  </si>
-  <si>
-    <t>Wai Hin Phyo</t>
-  </si>
-  <si>
-    <t>Hicham Charkaoui</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mohamed Shaheer Mohamed Laffir </t>
-  </si>
-  <si>
-    <t>Antony Kamau Kageche</t>
-  </si>
-  <si>
-    <t>Abdulrashid Byarugaba </t>
-  </si>
-  <si>
-    <t>Justine Tiangson Clave</t>
-  </si>
-  <si>
-    <t>Harikaran Seenithamby</t>
-  </si>
-  <si>
-    <t>Wycliffe Mushori</t>
-  </si>
-  <si>
-    <t>Peter Nganga Kamau</t>
-  </si>
-  <si>
-    <t>Sumesh Soman</t>
-  </si>
-  <si>
-    <t>Muhammed Ashiq Mohamed Mumtaz</t>
-  </si>
-  <si>
-    <t>Arvin Clyde D.Crisme</t>
-  </si>
-  <si>
-    <t>Gary John Packer</t>
-  </si>
-  <si>
-    <t>Ifras Mohammed</t>
-  </si>
-  <si>
-    <t>Alby Manchandiyil Antony</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ifran Ansari </t>
-  </si>
-  <si>
-    <t>Piratheepan Thiyagarasa</t>
-  </si>
-  <si>
-    <t>Moustafa Hassan Ibrahim Elsayyad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Harsha Shetty </t>
-  </si>
-  <si>
-    <t>Kevin Carl Enriquez Serrano</t>
-  </si>
-  <si>
-    <t>Romie Ross Tamayo Eleosida</t>
-  </si>
-  <si>
-    <t>Quennan Carandang Cuesta</t>
-  </si>
-  <si>
-    <t>Lester John Fuentes Monter</t>
-  </si>
-  <si>
-    <t>Neil Jhon Sabile Ramos</t>
-  </si>
-  <si>
-    <t>Kim Harvey Cuevas Ayag</t>
-  </si>
-  <si>
-    <t>Nelson Jr Ybut Sancho</t>
-  </si>
-  <si>
-    <t>Rolly Miano Valdez</t>
-  </si>
-  <si>
-    <t>Daniel Bacolcol Orquiza</t>
-  </si>
-  <si>
-    <t>Roby Chua Malinao</t>
-  </si>
-  <si>
-    <t>Lorence Cardenas Cabales</t>
-  </si>
-  <si>
-    <t>Emmanuel Richard Marasigan Velasco</t>
-  </si>
-  <si>
-    <t>Michael Jorge Toscano Masaoy</t>
-  </si>
-  <si>
-    <t>Jeffrey De Vera Cabico</t>
-  </si>
-  <si>
-    <t>Joe Peter Angustia Pimentel</t>
-  </si>
-  <si>
-    <t>Mark Roentgen Macatangay Delen</t>
-  </si>
-  <si>
-    <t>Arjay Imperial Gabarda</t>
-  </si>
-  <si>
-    <t>Noey Francisco Canonizado</t>
-  </si>
-  <si>
-    <t>Omar Zaki Saad Abdel Nabi</t>
-  </si>
-  <si>
-    <t>Abdul Rehman Mohammed Abdul Mohammed</t>
-  </si>
-  <si>
-    <t>Christian Merck Morada Martija</t>
-  </si>
-  <si>
-    <t>Imesha Rashmi Mudannayaka Mudannayakage</t>
-  </si>
-  <si>
-    <t>Sajith Dulanjana Kumara Rathnayaka Mudiyanselage</t>
-  </si>
-  <si>
-    <t>Thisura Kaumal Wijesinghe</t>
-  </si>
-  <si>
-    <t>Shanel Rukshan Perera Kurana Patabendige</t>
-  </si>
-  <si>
-    <t>Abeykoon Mudiyanselage Sasitha Dinushka Abeykoon</t>
-  </si>
-  <si>
-    <t>Jerusha Anns Philip</t>
+    <t>Justine Angwenyi Momanyi</t>
   </si>
   <si>
     <t>Management</t>
@@ -1590,7 +1593,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yy;@"/>
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1618,6 +1621,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1680,7 +1689,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1696,6 +1705,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2090,7 +2102,7 @@
         <v>245</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -2150,7 +2162,7 @@
         <v>248</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>232</v>
@@ -2172,7 +2184,7 @@
         <v>249</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>232</v>
@@ -2214,7 +2226,7 @@
         <v>251</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>232</v>
@@ -2236,7 +2248,7 @@
         <v>252</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>232</v>
@@ -2278,7 +2290,7 @@
         <v>251</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>232</v>
@@ -2300,7 +2312,7 @@
         <v>251</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -2337,10 +2349,10 @@
         <v>302</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>232</v>
@@ -2362,7 +2374,7 @@
         <v>251</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>232</v>
@@ -2404,7 +2416,7 @@
         <v>255</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>232</v>
@@ -2426,7 +2438,7 @@
         <v>256</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>232</v>
@@ -2448,7 +2460,7 @@
         <v>248</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>232</v>
@@ -2470,7 +2482,7 @@
         <v>255</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>232</v>
@@ -2492,7 +2504,7 @@
         <v>248</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>232</v>
@@ -2554,7 +2566,7 @@
         <v>252</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>232</v>
@@ -2576,7 +2588,7 @@
         <v>249</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>232</v>
@@ -2658,7 +2670,7 @@
         <v>248</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>232</v>
@@ -2700,7 +2712,7 @@
         <v>249</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>232</v>
@@ -2782,7 +2794,7 @@
         <v>255</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>232</v>
@@ -2804,7 +2816,7 @@
         <v>259</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>232</v>
@@ -2846,7 +2858,7 @@
         <v>252</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>232</v>
@@ -2888,7 +2900,7 @@
         <v>253</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>232</v>
@@ -2910,7 +2922,7 @@
         <v>253</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>232</v>
@@ -3172,7 +3184,7 @@
         <v>251</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>232</v>
@@ -3194,7 +3206,7 @@
         <v>245</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E55" s="1"/>
       <c r="F55" s="1"/>
@@ -3234,7 +3246,7 @@
         <v>264</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>232</v>
@@ -3256,7 +3268,7 @@
         <v>253</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>232</v>
@@ -3275,10 +3287,10 @@
         <v>347</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>232</v>
@@ -3300,7 +3312,7 @@
         <v>252</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>232</v>
@@ -3362,7 +3374,7 @@
         <v>256</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>232</v>
@@ -3384,7 +3396,7 @@
         <v>249</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>232</v>
@@ -3526,7 +3538,7 @@
         <v>259</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>232</v>
@@ -3588,7 +3600,7 @@
         <v>248</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>232</v>
@@ -3630,7 +3642,7 @@
         <v>253</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>232</v>
@@ -3652,7 +3664,7 @@
         <v>264</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>232</v>
@@ -3674,7 +3686,7 @@
         <v>268</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>232</v>
@@ -3716,7 +3728,7 @@
         <v>252</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>232</v>
@@ -3738,7 +3750,7 @@
         <v>252</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>232</v>
@@ -3780,7 +3792,7 @@
         <v>251</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E83" s="1"/>
       <c r="F83" s="1"/>
@@ -3920,7 +3932,7 @@
         <v>248</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E90" s="1" t="s">
         <v>232</v>
@@ -3962,7 +3974,7 @@
         <v>249</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>232</v>
@@ -4144,7 +4156,7 @@
         <v>268</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>232</v>
@@ -4163,7 +4175,7 @@
         <v>390</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="D102" s="1" t="s">
         <v>263</v>
@@ -4186,7 +4198,7 @@
         <v>248</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>232</v>
@@ -4248,7 +4260,7 @@
         <v>248</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E106" s="1" t="s">
         <v>232</v>
@@ -4267,7 +4279,7 @@
         <v>395</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D107" s="1" t="s">
         <v>254</v>
@@ -4292,7 +4304,7 @@
         <v>252</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>508</v>
+        <v>254</v>
       </c>
       <c r="E108" s="1" t="s">
         <v>232</v>
@@ -4314,7 +4326,7 @@
         <v>249</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E109" s="1" t="s">
         <v>232</v>
@@ -4329,14 +4341,14 @@
       <c r="A110" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B110" s="1" t="s">
-        <v>398</v>
+      <c r="B110" s="1" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="D110" s="1" t="s">
-        <v>254</v>
+      <c r="D110" s="1" t="e">
+        <v>#N/A</v>
       </c>
       <c r="E110" s="1"/>
       <c r="F110" s="1"/>
@@ -4350,7 +4362,7 @@
         <v>113</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>246</v>
@@ -4370,13 +4382,13 @@
         <v>114</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E112" s="1"/>
       <c r="F112" s="1"/>
@@ -4390,13 +4402,13 @@
         <v>115</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E113" s="1"/>
       <c r="F113" s="1"/>
@@ -4410,7 +4422,7 @@
         <v>116</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>254</v>
@@ -4430,13 +4442,13 @@
         <v>117</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>259</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E115" s="1" t="s">
         <v>232</v>
@@ -4452,7 +4464,7 @@
         <v>118</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>269</v>
@@ -4472,7 +4484,7 @@
         <v>119</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>261</v>
@@ -4492,7 +4504,7 @@
         <v>120</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>258</v>
@@ -4512,7 +4524,7 @@
         <v>121</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>260</v>
@@ -4532,7 +4544,7 @@
         <v>122</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>269</v>
@@ -4552,13 +4564,13 @@
         <v>123</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>255</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E121" s="1" t="s">
         <v>232</v>
@@ -4574,7 +4586,7 @@
         <v>124</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>265</v>
@@ -4594,13 +4606,13 @@
         <v>125</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>270</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E123" s="1" t="s">
         <v>232</v>
@@ -4616,7 +4628,7 @@
         <v>126</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>270</v>
@@ -4636,7 +4648,7 @@
         <v>127</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>265</v>
@@ -4656,13 +4668,13 @@
         <v>128</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>256</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E126" s="1" t="s">
         <v>232</v>
@@ -4678,7 +4690,7 @@
         <v>129</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>254</v>
@@ -4698,13 +4710,13 @@
         <v>130</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
@@ -4718,13 +4730,13 @@
         <v>131</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>250</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
@@ -4738,7 +4750,7 @@
         <v>132</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>271</v>
@@ -4758,13 +4770,13 @@
         <v>133</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
@@ -4778,13 +4790,13 @@
         <v>134</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>253</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E132" s="1" t="s">
         <v>232</v>
@@ -4800,7 +4812,7 @@
         <v>135</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>254</v>
@@ -4820,7 +4832,7 @@
         <v>136</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>265</v>
@@ -4840,13 +4852,13 @@
         <v>137</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>252</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E135" s="1" t="s">
         <v>232</v>
@@ -4862,7 +4874,7 @@
         <v>138</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>247</v>
@@ -4882,13 +4894,13 @@
         <v>139</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>264</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E137" s="1" t="s">
         <v>232</v>
@@ -4904,7 +4916,7 @@
         <v>140</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>257</v>
@@ -4924,13 +4936,13 @@
         <v>141</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>268</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E139" s="1" t="s">
         <v>232</v>
@@ -4946,7 +4958,7 @@
         <v>142</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>247</v>
@@ -4966,7 +4978,7 @@
         <v>143</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>261</v>
@@ -4986,7 +4998,7 @@
         <v>144</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>257</v>
@@ -5006,7 +5018,7 @@
         <v>145</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C143" s="1">
         <v>0</v>
@@ -5026,13 +5038,13 @@
         <v>146</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>249</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E144" s="1" t="s">
         <v>232</v>
@@ -5048,7 +5060,7 @@
         <v>147</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>257</v>
@@ -5068,7 +5080,7 @@
         <v>148</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>257</v>
@@ -5088,7 +5100,7 @@
         <v>149</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>257</v>
@@ -5108,7 +5120,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>255</v>
@@ -5128,13 +5140,13 @@
         <v>151</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>255</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E149" s="1" t="s">
         <v>232</v>
@@ -5150,7 +5162,7 @@
         <v>152</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>261</v>
@@ -5170,13 +5182,13 @@
         <v>153</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>264</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E151" s="1" t="s">
         <v>232</v>
@@ -5192,7 +5204,7 @@
         <v>154</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>254</v>
@@ -5214,13 +5226,13 @@
         <v>155</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E153" s="1"/>
       <c r="F153" s="1"/>
@@ -5234,13 +5246,13 @@
         <v>156</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E154" s="1"/>
       <c r="F154" s="1"/>
@@ -5254,13 +5266,13 @@
         <v>157</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>259</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E155" s="1" t="s">
         <v>232</v>
@@ -5276,13 +5288,13 @@
         <v>158</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>264</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E156" s="1" t="s">
         <v>232</v>
@@ -5298,7 +5310,7 @@
         <v>159</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>269</v>
@@ -5318,7 +5330,7 @@
         <v>160</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>254</v>
@@ -5340,13 +5352,13 @@
         <v>161</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>259</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E159" s="1" t="s">
         <v>232</v>
@@ -5362,13 +5374,13 @@
         <v>162</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E160" s="1" t="s">
         <v>232</v>
@@ -5384,13 +5396,13 @@
         <v>163</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>256</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E161" s="1" t="s">
         <v>232</v>
@@ -5406,7 +5418,7 @@
         <v>164</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>262</v>
@@ -5426,7 +5438,7 @@
         <v>165</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>265</v>
@@ -5446,7 +5458,7 @@
         <v>166</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>268</v>
@@ -5468,7 +5480,7 @@
         <v>167</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>254</v>
@@ -5488,7 +5500,7 @@
         <v>168</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>247</v>
@@ -5508,7 +5520,7 @@
         <v>169</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>268</v>
@@ -5528,7 +5540,7 @@
         <v>170</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>254</v>
@@ -5548,7 +5560,7 @@
         <v>171</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>265</v>
@@ -5568,7 +5580,7 @@
         <v>172</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>247</v>
@@ -5588,7 +5600,7 @@
         <v>173</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>252</v>
@@ -5610,13 +5622,13 @@
         <v>174</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D172" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E172" s="1"/>
       <c r="F172" s="1"/>
@@ -5630,7 +5642,7 @@
         <v>175</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>247</v>
@@ -5650,13 +5662,13 @@
         <v>176</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>272</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E174" s="1"/>
       <c r="F174" s="1"/>
@@ -5670,7 +5682,7 @@
         <v>177</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>257</v>
@@ -5690,7 +5702,7 @@
         <v>178</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>257</v>
@@ -5710,13 +5722,13 @@
         <v>179</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>255</v>
       </c>
       <c r="D177" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E177" s="1" t="s">
         <v>232</v>
@@ -5732,7 +5744,7 @@
         <v>180</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>259</v>
@@ -5752,13 +5764,13 @@
         <v>181</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>255</v>
       </c>
       <c r="D179" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E179" s="1" t="s">
         <v>232</v>
@@ -5774,13 +5786,13 @@
         <v>182</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>264</v>
       </c>
       <c r="D180" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E180" s="1" t="s">
         <v>232</v>
@@ -5796,13 +5808,13 @@
         <v>183</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>268</v>
       </c>
       <c r="D181" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E181" s="1" t="s">
         <v>232</v>
@@ -5818,13 +5830,13 @@
         <v>184</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D182" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E182" s="1"/>
       <c r="F182" s="1"/>
@@ -5838,13 +5850,13 @@
         <v>185</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>262</v>
       </c>
       <c r="D183" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E183" s="1"/>
       <c r="F183" s="1"/>
@@ -5858,7 +5870,7 @@
         <v>186</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C184" s="1" t="s">
         <v>251</v>
@@ -5880,13 +5892,13 @@
         <v>187</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C185" s="1" t="s">
         <v>273</v>
       </c>
       <c r="D185" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E185" s="1"/>
       <c r="F185" s="1"/>
@@ -5900,7 +5912,7 @@
         <v>188</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>261</v>
@@ -5920,13 +5932,13 @@
         <v>189</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D187" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E187" s="1" t="s">
         <v>232</v>
@@ -5942,13 +5954,13 @@
         <v>190</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C188" s="1" t="s">
         <v>256</v>
       </c>
       <c r="D188" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E188" s="1" t="s">
         <v>232</v>
@@ -5964,7 +5976,7 @@
         <v>191</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>274</v>
@@ -5984,7 +5996,7 @@
         <v>192</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C190" s="1" t="s">
         <v>275</v>
@@ -6004,13 +6016,13 @@
         <v>193</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D191" s="1" t="s">
-        <v>508</v>
+        <v>254</v>
       </c>
       <c r="E191" s="1" t="s">
         <v>232</v>
@@ -6026,13 +6038,13 @@
         <v>194</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C192" s="1" t="s">
         <v>256</v>
       </c>
       <c r="D192" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E192" s="1" t="s">
         <v>232</v>
@@ -6048,13 +6060,13 @@
         <v>195</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C193" s="1" t="s">
         <v>249</v>
       </c>
       <c r="D193" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E193" s="1" t="s">
         <v>232</v>
@@ -6070,13 +6082,13 @@
         <v>196</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C194" s="1" t="s">
         <v>266</v>
       </c>
       <c r="D194" s="1" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E194" s="1" t="s">
         <v>232</v>
@@ -6092,7 +6104,7 @@
         <v>197</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C195" s="1" t="s">
         <v>247</v>
@@ -6112,7 +6124,7 @@
         <v>198</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C196" s="1" t="s">
         <v>266</v>
@@ -6134,7 +6146,7 @@
         <v>199</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C197" s="1" t="s">
         <v>247</v>
@@ -6154,7 +6166,7 @@
         <v>200</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>262</v>
@@ -6174,13 +6186,13 @@
         <v>201</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C199" s="1" t="s">
         <v>248</v>
       </c>
       <c r="D199" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E199" s="1" t="s">
         <v>232</v>
@@ -6196,13 +6208,13 @@
         <v>202</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C200" s="1" t="s">
         <v>264</v>
       </c>
       <c r="D200" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E200" s="1" t="s">
         <v>232</v>
@@ -6218,7 +6230,7 @@
         <v>203</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C201" s="1" t="s">
         <v>260</v>
@@ -6238,7 +6250,7 @@
         <v>204</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C202" s="1" t="s">
         <v>247</v>
@@ -6258,13 +6270,13 @@
         <v>205</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C203" s="1" t="s">
         <v>249</v>
       </c>
       <c r="D203" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E203" s="1" t="s">
         <v>232</v>
@@ -6280,13 +6292,13 @@
         <v>206</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C204" s="1" t="s">
         <v>249</v>
       </c>
       <c r="D204" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E204" s="1" t="s">
         <v>232</v>
@@ -6302,7 +6314,7 @@
         <v>207</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C205" s="1" t="s">
         <v>266</v>
@@ -6324,7 +6336,7 @@
         <v>208</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C206" s="1" t="s">
         <v>262</v>
@@ -6344,13 +6356,13 @@
         <v>209</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C207" s="1" t="s">
         <v>264</v>
       </c>
       <c r="D207" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E207" s="1" t="s">
         <v>232</v>
@@ -6366,13 +6378,13 @@
         <v>210</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C208" s="1" t="s">
         <v>266</v>
       </c>
       <c r="D208" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E208" s="1" t="s">
         <v>232</v>
@@ -6388,13 +6400,13 @@
         <v>211</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C209" s="1" t="s">
         <v>253</v>
       </c>
       <c r="D209" s="1" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="E209" s="1" t="s">
         <v>232</v>
@@ -6410,13 +6422,13 @@
         <v>212</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C210" s="1" t="s">
         <v>250</v>
       </c>
       <c r="D210" s="1" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="E210" s="1"/>
       <c r="F210" s="1"/>
@@ -6430,13 +6442,13 @@
         <v>213</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C211" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D211" s="1" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E211" s="1"/>
       <c r="F211" s="1"/>
@@ -6450,7 +6462,7 @@
         <v>214</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C212" s="1" t="s">
         <v>263</v>
@@ -6470,7 +6482,7 @@
         <v>215</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C213" s="1" t="s">
         <v>274</v>
@@ -6490,13 +6502,13 @@
         <v>216</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C214" s="1" t="s">
         <v>256</v>
       </c>
       <c r="D214" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E214" s="1" t="s">
         <v>232</v>
@@ -6512,7 +6524,7 @@
         <v>217</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C215" s="1" t="s">
         <v>263</v>
@@ -6532,13 +6544,13 @@
         <v>218</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C216" s="1" t="s">
         <v>268</v>
       </c>
       <c r="D216" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E216" s="1" t="s">
         <v>232</v>
@@ -6554,13 +6566,13 @@
         <v>219</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C217" s="1" t="s">
         <v>268</v>
       </c>
       <c r="D217" s="1" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="E217" s="1" t="s">
         <v>232</v>
@@ -6576,7 +6588,7 @@
         <v>220</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C218" s="1" t="s">
         <v>246</v>
@@ -6595,14 +6607,14 @@
       <c r="A219" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B219" s="1">
-        <v>0</v>
-      </c>
-      <c r="C219" s="1">
-        <v>0</v>
-      </c>
-      <c r="D219" s="1">
-        <v>0</v>
+      <c r="B219" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="C219" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D219" s="1" t="s">
+        <v>247</v>
       </c>
       <c r="E219" s="1"/>
       <c r="F219" s="1"/>
@@ -6615,14 +6627,14 @@
       <c r="A220" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B220" s="1">
-        <v>0</v>
-      </c>
-      <c r="C220" s="1">
-        <v>0</v>
-      </c>
-      <c r="D220" s="1">
-        <v>0</v>
+      <c r="B220" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="C220" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="D220" s="1" t="s">
+        <v>510</v>
       </c>
       <c r="E220" s="1"/>
       <c r="F220" s="1"/>
@@ -7452,7 +7464,7 @@
         <v>302</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D14" s="1">
         <v>0</v>
@@ -9866,7 +9878,7 @@
         <v>347</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D59" s="1">
         <v>0</v>
@@ -12160,7 +12172,7 @@
         <v>390</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="D102" s="1">
         <v>0</v>
@@ -12462,7 +12474,7 @@
         <v>395</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D107" s="1">
         <v>0</v>
@@ -12634,8 +12646,8 @@
       <c r="A110" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B110" s="1" t="s">
-        <v>398</v>
+      <c r="B110" s="1" t="e">
+        <v>#N/A</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>247</v>
@@ -12677,7 +12689,7 @@
         <v>113</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>246</v>
@@ -12719,7 +12731,7 @@
         <v>114</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>251</v>
@@ -12761,7 +12773,7 @@
         <v>115</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>251</v>
@@ -12803,7 +12815,7 @@
         <v>116</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>254</v>
@@ -12845,7 +12857,7 @@
         <v>117</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>259</v>
@@ -12929,7 +12941,7 @@
         <v>118</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C116" s="1" t="s">
         <v>269</v>
@@ -12971,7 +12983,7 @@
         <v>119</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C117" s="1" t="s">
         <v>261</v>
@@ -13013,7 +13025,7 @@
         <v>120</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>258</v>
@@ -13055,7 +13067,7 @@
         <v>121</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>260</v>
@@ -13097,7 +13109,7 @@
         <v>122</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>269</v>
@@ -13139,7 +13151,7 @@
         <v>123</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C121" s="1" t="s">
         <v>255</v>
@@ -13217,7 +13229,7 @@
         <v>124</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>265</v>
@@ -13259,7 +13271,7 @@
         <v>125</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>270</v>
@@ -13301,7 +13313,7 @@
         <v>126</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>270</v>
@@ -13343,7 +13355,7 @@
         <v>127</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>265</v>
@@ -13385,7 +13397,7 @@
         <v>128</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>256</v>
@@ -13465,7 +13477,7 @@
         <v>129</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>254</v>
@@ -13507,7 +13519,7 @@
         <v>130</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>251</v>
@@ -13549,7 +13561,7 @@
         <v>131</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>250</v>
@@ -13591,7 +13603,7 @@
         <v>132</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>271</v>
@@ -13633,7 +13645,7 @@
         <v>133</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>251</v>
@@ -13675,7 +13687,7 @@
         <v>134</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>253</v>
@@ -13759,7 +13771,7 @@
         <v>135</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>254</v>
@@ -13801,7 +13813,7 @@
         <v>136</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>265</v>
@@ -13843,7 +13855,7 @@
         <v>137</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>252</v>
@@ -13913,7 +13925,7 @@
         <v>138</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>247</v>
@@ -13955,7 +13967,7 @@
         <v>139</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>264</v>
@@ -14033,7 +14045,7 @@
         <v>140</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>257</v>
@@ -14075,7 +14087,7 @@
         <v>141</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>268</v>
@@ -14159,7 +14171,7 @@
         <v>142</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>247</v>
@@ -14201,7 +14213,7 @@
         <v>143</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>261</v>
@@ -14243,7 +14255,7 @@
         <v>144</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>257</v>
@@ -14285,7 +14297,7 @@
         <v>145</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C143" s="1">
         <v>0</v>
@@ -14327,7 +14339,7 @@
         <v>146</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>249</v>
@@ -14411,7 +14423,7 @@
         <v>147</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>257</v>
@@ -14453,7 +14465,7 @@
         <v>148</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>257</v>
@@ -14495,7 +14507,7 @@
         <v>149</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>257</v>
@@ -14537,7 +14549,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>255</v>
@@ -14579,7 +14591,7 @@
         <v>151</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>255</v>
@@ -14663,7 +14675,7 @@
         <v>152</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>261</v>
@@ -14705,7 +14717,7 @@
         <v>153</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>264</v>
@@ -14773,7 +14785,7 @@
         <v>154</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>254</v>
@@ -14815,7 +14827,7 @@
         <v>155</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>251</v>
@@ -14857,7 +14869,7 @@
         <v>156</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>251</v>
@@ -14899,7 +14911,7 @@
         <v>157</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>259</v>
@@ -14967,7 +14979,7 @@
         <v>158</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>264</v>
@@ -15009,7 +15021,7 @@
         <v>159</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>269</v>
@@ -15051,7 +15063,7 @@
         <v>160</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>254</v>
@@ -15093,7 +15105,7 @@
         <v>161</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>259</v>
@@ -15175,7 +15187,7 @@
         <v>162</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>251</v>
@@ -15217,7 +15229,7 @@
         <v>163</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>256</v>
@@ -15297,7 +15309,7 @@
         <v>164</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>262</v>
@@ -15339,7 +15351,7 @@
         <v>165</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>265</v>
@@ -15381,7 +15393,7 @@
         <v>166</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>268</v>
@@ -15423,7 +15435,7 @@
         <v>167</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>254</v>
@@ -15465,7 +15477,7 @@
         <v>168</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>247</v>
@@ -15507,7 +15519,7 @@
         <v>169</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>268</v>
@@ -15549,7 +15561,7 @@
         <v>170</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>254</v>
@@ -15591,7 +15603,7 @@
         <v>171</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>265</v>
@@ -15633,7 +15645,7 @@
         <v>172</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>247</v>
@@ -15675,7 +15687,7 @@
         <v>173</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>252</v>
@@ -15717,7 +15729,7 @@
         <v>174</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>251</v>
@@ -15759,7 +15771,7 @@
         <v>175</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>247</v>
@@ -15801,7 +15813,7 @@
         <v>176</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>272</v>
@@ -15843,7 +15855,7 @@
         <v>177</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>257</v>
@@ -15885,7 +15897,7 @@
         <v>178</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>257</v>
@@ -15927,7 +15939,7 @@
         <v>179</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>255</v>
@@ -16013,7 +16025,7 @@
         <v>180</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>259</v>
@@ -16055,7 +16067,7 @@
         <v>181</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>255</v>
@@ -16125,7 +16137,7 @@
         <v>182</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>264</v>
@@ -16203,7 +16215,7 @@
         <v>183</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>268</v>
@@ -16275,7 +16287,7 @@
         <v>184</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>251</v>
@@ -16317,7 +16329,7 @@
         <v>185</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>262</v>
@@ -16359,7 +16371,7 @@
         <v>186</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="C184" s="1" t="s">
         <v>251</v>
@@ -16401,7 +16413,7 @@
         <v>187</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C185" s="1" t="s">
         <v>273</v>
@@ -16443,7 +16455,7 @@
         <v>188</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>261</v>
@@ -16485,7 +16497,7 @@
         <v>189</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>251</v>
@@ -16527,7 +16539,7 @@
         <v>190</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C188" s="1" t="s">
         <v>256</v>
@@ -16607,7 +16619,7 @@
         <v>191</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>274</v>
@@ -16649,7 +16661,7 @@
         <v>192</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="C190" s="1" t="s">
         <v>275</v>
@@ -16691,10 +16703,10 @@
         <v>193</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C191" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D191" s="1">
         <v>21</v>
@@ -16775,7 +16787,7 @@
         <v>194</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="C192" s="1" t="s">
         <v>256</v>
@@ -16861,7 +16873,7 @@
         <v>195</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="C193" s="1" t="s">
         <v>249</v>
@@ -16933,7 +16945,7 @@
         <v>196</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C194" s="1" t="s">
         <v>266</v>
@@ -16975,7 +16987,7 @@
         <v>197</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="C195" s="1" t="s">
         <v>247</v>
@@ -17017,7 +17029,7 @@
         <v>198</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="C196" s="1" t="s">
         <v>266</v>
@@ -17059,7 +17071,7 @@
         <v>199</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="C197" s="1" t="s">
         <v>247</v>
@@ -17101,7 +17113,7 @@
         <v>200</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>262</v>
@@ -17143,7 +17155,7 @@
         <v>201</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C199" s="1" t="s">
         <v>248</v>
@@ -17235,7 +17247,7 @@
         <v>202</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C200" s="1" t="s">
         <v>264</v>
@@ -17319,7 +17331,7 @@
         <v>203</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C201" s="1" t="s">
         <v>260</v>
@@ -17361,7 +17373,7 @@
         <v>204</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="C202" s="1" t="s">
         <v>247</v>
@@ -17403,7 +17415,7 @@
         <v>205</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C203" s="1" t="s">
         <v>249</v>
@@ -17487,7 +17499,7 @@
         <v>206</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C204" s="1" t="s">
         <v>249</v>
@@ -17565,7 +17577,7 @@
         <v>207</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="C205" s="1" t="s">
         <v>266</v>
@@ -17607,7 +17619,7 @@
         <v>208</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="C206" s="1" t="s">
         <v>262</v>
@@ -17649,7 +17661,7 @@
         <v>209</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="C207" s="1" t="s">
         <v>264</v>
@@ -17707,7 +17719,7 @@
         <v>210</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="C208" s="1" t="s">
         <v>266</v>
@@ -17777,7 +17789,7 @@
         <v>211</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C209" s="1" t="s">
         <v>253</v>
@@ -17861,7 +17873,7 @@
         <v>212</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C210" s="1" t="s">
         <v>250</v>
@@ -17903,7 +17915,7 @@
         <v>213</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="C211" s="1" t="s">
         <v>251</v>
@@ -17945,7 +17957,7 @@
         <v>214</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="C212" s="1" t="s">
         <v>263</v>
@@ -17987,7 +17999,7 @@
         <v>215</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="C213" s="1" t="s">
         <v>274</v>
@@ -18029,7 +18041,7 @@
         <v>216</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="C214" s="1" t="s">
         <v>256</v>
@@ -18107,7 +18119,7 @@
         <v>217</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C215" s="1" t="s">
         <v>263</v>
@@ -18149,7 +18161,7 @@
         <v>218</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C216" s="1" t="s">
         <v>268</v>
@@ -18233,7 +18245,7 @@
         <v>219</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="C217" s="1" t="s">
         <v>268</v>
@@ -18317,7 +18329,7 @@
         <v>220</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="C218" s="1" t="s">
         <v>246</v>
@@ -18358,11 +18370,11 @@
       <c r="A219" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B219" s="1">
-        <v>0</v>
-      </c>
-      <c r="C219" s="1">
-        <v>0</v>
+      <c r="B219" s="1" t="s">
+        <v>506</v>
+      </c>
+      <c r="C219" s="1" t="s">
+        <v>247</v>
       </c>
       <c r="D219" s="1">
         <v>0</v>
@@ -18400,14 +18412,14 @@
       <c r="A220" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B220" s="1">
-        <v>0</v>
-      </c>
-      <c r="C220" s="1">
-        <v>0</v>
+      <c r="B220" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="C220" s="1" t="s">
+        <v>266</v>
       </c>
       <c r="D220" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E220" s="6"/>
       <c r="F220" s="6"/>
@@ -18426,7 +18438,9 @@
       <c r="S220" s="6"/>
       <c r="T220" s="6"/>
       <c r="U220" s="6"/>
-      <c r="V220" s="6"/>
+      <c r="V220" s="11">
+        <v>46301</v>
+      </c>
       <c r="W220" s="6"/>
       <c r="X220" s="6"/>
       <c r="Y220" s="6"/>

</xml_diff>